<commit_message>
Refactor CSS styles and add autocomplete functionality
- Refactor CSS styles in style.css to improve readability and organization.
- Add autocomplete functionality to the course input field in script.js to provide suggestions for course titles based on user input.
</commit_message>
<xml_diff>
--- a/api/asset/mid-term-exam-schedule_notice-board_sose_243.xlsx
+++ b/api/asset/mid-term-exam-schedule_notice-board_sose_243.xlsx
@@ -6884,7 +6884,7 @@
         <v>352</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="148" customHeight="1" ht="28.5">
       <c r="A148" s="5" t="s">
         <v>69</v>
       </c>
@@ -6910,7 +6910,7 @@
         <v>354</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="149" customHeight="1" ht="28.5">
       <c r="A149" s="5" t="s">
         <v>69</v>
       </c>
@@ -6936,7 +6936,7 @@
         <v>357</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="150" customHeight="1" ht="28.5">
       <c r="A150" s="5" t="s">
         <v>69</v>
       </c>
@@ -6962,7 +6962,7 @@
         <v>359</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="151" customHeight="1" ht="28.5">
       <c r="A151" s="5" t="s">
         <v>8</v>
       </c>
@@ -6988,7 +6988,7 @@
         <v>361</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="152" customHeight="1" ht="28.5">
       <c r="A152" s="5" t="s">
         <v>8</v>
       </c>
@@ -7014,7 +7014,7 @@
         <v>362</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="153" customHeight="1" ht="28.5">
       <c r="A153" s="5" t="s">
         <v>8</v>
       </c>
@@ -7040,7 +7040,7 @@
         <v>363</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="154" customHeight="1" ht="28.5">
       <c r="A154" s="5" t="s">
         <v>8</v>
       </c>
@@ -7066,7 +7066,7 @@
         <v>364</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="155" customHeight="1" ht="28.5">
       <c r="A155" s="5" t="s">
         <v>8</v>
       </c>
@@ -7092,7 +7092,7 @@
         <v>365</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="156" customHeight="1" ht="28.5">
       <c r="A156" s="5" t="s">
         <v>8</v>
       </c>
@@ -7118,7 +7118,7 @@
         <v>367</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="157" customHeight="1" ht="28.5">
       <c r="A157" s="5" t="s">
         <v>8</v>
       </c>
@@ -7144,7 +7144,7 @@
         <v>369</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="158" customHeight="1" ht="28.5">
       <c r="A158" s="5" t="s">
         <v>8</v>
       </c>
@@ -7170,7 +7170,7 @@
         <v>371</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="159" customHeight="1" ht="28.5">
       <c r="A159" s="5" t="s">
         <v>8</v>
       </c>
@@ -7196,7 +7196,7 @@
         <v>373</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="160" customHeight="1" ht="28.5">
       <c r="A160" s="5" t="s">
         <v>8</v>
       </c>
@@ -7222,7 +7222,7 @@
         <v>374</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="161" customHeight="1" ht="28.5">
       <c r="A161" s="5" t="s">
         <v>8</v>
       </c>
@@ -7248,7 +7248,7 @@
         <v>375</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="162" customHeight="1" ht="28.5">
       <c r="A162" s="5" t="s">
         <v>8</v>
       </c>
@@ -7274,7 +7274,7 @@
         <v>377</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="163" customHeight="1" ht="28.5">
       <c r="A163" s="5" t="s">
         <v>8</v>
       </c>
@@ -7300,7 +7300,7 @@
         <v>378</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="164" customHeight="1" ht="28.5">
       <c r="A164" s="5" t="s">
         <v>8</v>
       </c>
@@ -7326,7 +7326,7 @@
         <v>379</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="165" customHeight="1" ht="28.5">
       <c r="A165" s="5" t="s">
         <v>8</v>
       </c>
@@ -7352,7 +7352,7 @@
         <v>382</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="166" customHeight="1" ht="28.5">
       <c r="A166" s="5" t="s">
         <v>8</v>
       </c>
@@ -7404,7 +7404,7 @@
         <v>387</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="168" customHeight="1" ht="28.5">
       <c r="A168" s="5" t="s">
         <v>8</v>
       </c>
@@ -7430,7 +7430,7 @@
         <v>389</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="169" customHeight="1" ht="28.5">
       <c r="A169" s="5" t="s">
         <v>20</v>
       </c>
@@ -7456,7 +7456,7 @@
         <v>392</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="170" customHeight="1" ht="28.5">
       <c r="A170" s="5" t="s">
         <v>20</v>
       </c>
@@ -7508,7 +7508,7 @@
         <v>398</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="172" customHeight="1" ht="28.5">
       <c r="A172" s="5" t="s">
         <v>8</v>
       </c>
@@ -7534,7 +7534,7 @@
         <v>402</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="173" customHeight="1" ht="28.5">
       <c r="A173" s="5" t="s">
         <v>8</v>
       </c>
@@ -7560,7 +7560,7 @@
         <v>404</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="174" customHeight="1" ht="28.5">
       <c r="A174" s="5" t="s">
         <v>8</v>
       </c>
@@ -7586,7 +7586,7 @@
         <v>405</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="175" customHeight="1" ht="28.5">
       <c r="A175" s="5" t="s">
         <v>8</v>
       </c>
@@ -7612,7 +7612,7 @@
         <v>406</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="176" customHeight="1" ht="28.5">
       <c r="A176" s="5" t="s">
         <v>8</v>
       </c>
@@ -7638,7 +7638,7 @@
         <v>408</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="177" customHeight="1" ht="28.5">
       <c r="A177" s="5" t="s">
         <v>69</v>
       </c>
@@ -7664,7 +7664,7 @@
         <v>411</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="178" customHeight="1" ht="28.5">
       <c r="A178" s="5" t="s">
         <v>69</v>
       </c>
@@ -7690,7 +7690,7 @@
         <v>412</v>
       </c>
     </row>
-    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="17.25">
+    <row x14ac:dyDescent="0.25" r="179" customHeight="1" ht="28.5">
       <c r="A179" s="5" t="s">
         <v>8</v>
       </c>

</xml_diff>